<commit_message>
chore(jdt): jdt mis a jour pour la journée
</commit_message>
<xml_diff>
--- a/T-P_320-pe84djb-JDT.xlsx
+++ b/T-P_320-pe84djb-JDT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pe84djb\Documents\GitHub\Projet-320-ShootMeUp-YFS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E14DF893-1075-48C1-88A4-8D8D45D6A7FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1491FBB-39E9-4382-AF36-FA04A8589BF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="29">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -131,6 +131,12 @@
   </si>
   <si>
     <t>yohannf-222/Projet-320-ShootMeUp-YFS: Une version alternative de space invaders</t>
+  </si>
+  <si>
+    <t>organisation</t>
+  </si>
+  <si>
+    <t>Nous testons gitjournal (remplacé par ce jdt), je change des fichiers dans le repo (cdc).</t>
   </si>
 </sst>
 </file>
@@ -944,7 +950,7 @@
       </c>
       <c r="B7" s="37"/>
       <c r="C7" s="8">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>25</v>
@@ -952,10 +958,16 @@
       <c r="E7" s="25"/>
     </row>
     <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7"/>
+      <c r="A8" s="7" t="s">
+        <v>27</v>
+      </c>
       <c r="B8" s="37"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="9"/>
+      <c r="C8" s="8">
+        <v>35</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>28</v>
+      </c>
       <c r="E8" s="8"/>
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -2027,7 +2039,7 @@
       <c r="B155" s="28"/>
       <c r="C155" s="15">
         <f>MROUND(SUM(C6:C154) /60,0.2)</f>
-        <v>2.4000000000000004</v>
+        <v>3</v>
       </c>
       <c r="D155" s="16"/>
       <c r="E155" s="17"/>

</xml_diff>